<commit_message>
Framework changes - Add Proper Page Class with Base class and Excel test data file
</commit_message>
<xml_diff>
--- a/test-data/TestData.xlsx
+++ b/test-data/TestData.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Playwright Automation\Playwright_Learn_Framework\test-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30987AD1-9C4F-4B1F-A953-09A60AED49FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAE26A23-3549-414F-BCAE-41BEB723B9E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="guestmakepayment" sheetId="1" r:id="rId1"/>
-    <sheet name="logincredential" sheetId="2" r:id="rId2"/>
+    <sheet name="loginData" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="34">
   <si>
     <t>error</t>
   </si>
@@ -64,24 +64,12 @@
     <t>secret_sauce</t>
   </si>
   <si>
-    <t>success</t>
-  </si>
-  <si>
     <t>yes</t>
   </si>
   <si>
     <t>locked_out_user</t>
   </si>
   <si>
-    <t>problem_user</t>
-  </si>
-  <si>
-    <t>error_user</t>
-  </si>
-  <si>
-    <t>visual_user</t>
-  </si>
-  <si>
     <t>no</t>
   </si>
   <si>
@@ -92,14 +80,70 @@
   </si>
   <si>
     <t>11115555</t>
+  </si>
+  <si>
+    <t>scenario</t>
+  </si>
+  <si>
+    <t>valid_credential</t>
+  </si>
+  <si>
+    <t>username_missing</t>
+  </si>
+  <si>
+    <t>invalid_credential</t>
+  </si>
+  <si>
+    <t>password_missing</t>
+  </si>
+  <si>
+    <t>testname</t>
+  </si>
+  <si>
+    <t>summary</t>
+  </si>
+  <si>
+    <t>verify Error messages with invalid credentials.</t>
+  </si>
+  <si>
+    <t>Play-303</t>
+  </si>
+  <si>
+    <t>Play-304</t>
+  </si>
+  <si>
+    <t>verify Error messages with username missing in credentials.</t>
+  </si>
+  <si>
+    <t>Play-305</t>
+  </si>
+  <si>
+    <t>verify Error messages with password missing in credentials.</t>
+  </si>
+  <si>
+    <t>Play-306</t>
+  </si>
+  <si>
+    <t>comment</t>
+  </si>
+  <si>
+    <t>verify Login with valid credentials.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -127,9 +171,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -418,16 +463,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+      <c r="A1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="2" t="s">
         <v>4</v>
       </c>
     </row>
@@ -447,7 +492,7 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>7</v>
@@ -456,12 +501,12 @@
         <v>0</v>
       </c>
       <c r="D3" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>7</v>
@@ -470,12 +515,12 @@
         <v>0</v>
       </c>
       <c r="D4" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>7</v>
@@ -484,7 +529,7 @@
         <v>0</v>
       </c>
       <c r="D5" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -495,98 +540,122 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32791E77-9F60-42F8-AB59-732FF739E7B7}">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.88671875" customWidth="1"/>
-    <col min="2" max="2" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="53.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.5546875" customWidth="1"/>
+    <col min="5" max="5" width="14.5546875" customWidth="1"/>
+    <col min="6" max="6" width="20.44140625" customWidth="1"/>
+    <col min="7" max="7" width="33.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B1" t="s">
+      <c r="E1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="F1" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D2" t="s">
         <v>10</v>
       </c>
-      <c r="B2" t="s">
+      <c r="E2" t="s">
         <v>11</v>
       </c>
-      <c r="C2" t="s">
+      <c r="F2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
         <v>12</v>
       </c>
-      <c r="D2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>14</v>
-      </c>
       <c r="B3" t="s">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="C3" t="s">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="D3" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" t="s">
         <v>11</v>
       </c>
-      <c r="C4" t="s">
+      <c r="F4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
         <v>12</v>
       </c>
-      <c r="D4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>16</v>
-      </c>
       <c r="B5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D5" t="s">
+        <v>10</v>
+      </c>
+      <c r="E5" t="s">
         <v>11</v>
       </c>
-      <c r="C5" t="s">
-        <v>12</v>
-      </c>
-      <c r="D5" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>17</v>
-      </c>
-      <c r="B6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C6" t="s">
-        <v>12</v>
-      </c>
-      <c r="D6" t="s">
-        <v>18</v>
+      <c r="F5" t="s">
+        <v>22</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Change Framework folder structure
</commit_message>
<xml_diff>
--- a/test-data/TestData.xlsx
+++ b/test-data/TestData.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Automation\Playwright Automation\Playwright_Learn_Framework\test-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAE26A23-3549-414F-BCAE-41BEB723B9E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11427D0F-8C3E-43A1-98E1-492189569B12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="guestmakepayment" sheetId="1" r:id="rId1"/>
-    <sheet name="loginData" sheetId="2" r:id="rId2"/>
+    <sheet name="login" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>

</xml_diff>